<commit_message>
UI test changing the parameters
Changed the parameters to make the text larger than the window size
</commit_message>
<xml_diff>
--- a/Test_Log.xlsx
+++ b/Test_Log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Student\Documents\GitHub\angry-birds-clone-assignment-SundaysWithoutGod\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C04097E-D1FE-4564-A365-2B0C1C519245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BCE844-9FC9-4474-8780-BB5BBB9B5220}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F675273F-C51E-4954-B235-DAD390D71047}"/>
   </bookViews>
@@ -189,7 +189,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="54">
   <si>
     <t>Date:</t>
   </si>
@@ -385,6 +385,12 @@
   <si>
     <t>The UI text will be less than 
 the window screen</t>
+  </si>
+  <si>
+    <t>98b6503</t>
+  </si>
+  <si>
+    <t>Changed the parameters of size in the UI to be lar</t>
   </si>
 </sst>
 </file>
@@ -1318,7 +1324,9 @@
       <c r="B12" s="3">
         <v>46169</v>
       </c>
-      <c r="C12" s="9"/>
+      <c r="C12" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="D12" s="27" t="s">
         <v>50</v>
       </c>
@@ -1341,9 +1349,13 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B13" s="3"/>
+      <c r="B13" s="3">
+        <v>46169</v>
+      </c>
       <c r="C13" s="9"/>
-      <c r="D13" s="6"/>
+      <c r="D13" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="E13" s="9"/>
       <c r="F13" s="6"/>
       <c r="G13" s="9"/>

</xml_diff>